<commit_message>
expense details download function is working now
</commit_message>
<xml_diff>
--- a/backend/expense_details.xlsx
+++ b/backend/expense_details.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,18 +413,73 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Medicine</v>
+      </c>
+      <c r="B2">
+        <v>1000</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46000.229537037034</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="B3">
+        <v>1000</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45999.229537037034</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="B4">
+        <v>500</v>
+      </c>
+      <c r="C4" s="1">
+        <v>45999.229537037034</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>Rent</v>
       </c>
-      <c r="B2">
-        <v>40000</v>
-      </c>
-      <c r="C2" s="1">
-        <v>45484.229537037034</v>
+      <c r="B5">
+        <v>20000</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45998.229537037034</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Car Service</v>
+      </c>
+      <c r="B6">
+        <v>20000</v>
+      </c>
+      <c r="C6" s="1">
+        <v>45997.229537037034</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Wifi</v>
+      </c>
+      <c r="B7">
+        <v>15000</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45996.229537037034</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>